<commit_message>
feat(quick-260408-lbn): extend luban phase1 export for action/task/office
- add workbook and Luban define support for action, task, and office tables
- publish generated JSON outputs and index mappings on the existing phase1 pipeline
</commit_message>
<xml_diff>
--- a/data-authoring/excel/190_smoke_sample.xlsx
+++ b/data-authoring/excel/190_smoke_sample.xlsx
@@ -11,6 +11,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Faction" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="City" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Character" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Action" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1341,4 +1344,1132 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>display_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>category_id</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>ap_cost</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>energy_delta</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>target_type</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>effect_summary</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>required_permission_tags</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>allowed_identity_types</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>locked_reason</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>menu_order</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>hidden_when_locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>train</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>训练</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>成长</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-10</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>效果: 武艺历练 +6，压力 +3，功绩 +1</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>ruler|civil_official|military_officer|free_agent</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>当前身份不可执行</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>10</v>
+      </c>
+      <c r="L2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>读书</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>成长</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-8</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>效果: 智略历练 +6，压力 +2，名望 +1</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>ruler|civil_official|military_officer|free_agent</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>当前身份不可执行</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>20</v>
+      </c>
+      <c r="L3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>rest</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>休整</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>成长</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>20</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>效果: 精力 +20，压力 -12</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>ruler|civil_official|military_officer|free_agent</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>当前身份不可执行</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>30</v>
+      </c>
+      <c r="L4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>visit</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>拜访</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>关系</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-8</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>character</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>效果: 好感 +10，信任 +6，敬重 +2，戒备 -4</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>ruler|civil_official|military_officer|free_agent</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>当前身份不可执行</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>40</v>
+      </c>
+      <c r="L5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>inspect</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>巡察</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>政务</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-10</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>效果: 功绩 +5，政务历练 +4，压力 +4</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>ruler|civil_official|military_officer</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>当前身份不可执行</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>50</v>
+      </c>
+      <c r="L6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:U5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>issuer_character_id</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>issuer_role_tag</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>task_type</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>task_tags</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>min_office_tier</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>max_office_tier</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>objective_summary</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>duration_months</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>difficulty</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>progress_rule_id</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>success_condition</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>excellent_condition</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>base_rewards</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>bonus_rewards</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>fail_result</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>followup_tags</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>ui_priority</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>is_phase2_1_available</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>task_document_cleanup</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>整顿文书</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>cao_cao</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>ruler</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>清理积压案牍、统一文书格式，并补齐府署往来登记，使政务流转恢复秩序。</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>以读书与巡察配合整理文案，本月务求案牍无滞。</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>document_cleanup_admin</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>current_value:8</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>current_value:11</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>merit:7|fame:1|trust:1|success_note:案牍条理分明，曹操认为你足以承担更稳重的府署事务。</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>merit:3|fame:1|trust:1|success_note:文书积弊一并肃清，幕府上下对你的办事分寸更为放心。</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>merit_delta:0|fame_delta:0|trust_delta:-1|failure_note:文案仍有疏漏，上意虽未重责，但对你本月掌事的把握略生疑虑。</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>admin|personnel</t>
+        </is>
+      </c>
+      <c r="T2" t="n">
+        <v>100</v>
+      </c>
+      <c r="U2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>task_grain_audit</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>整理军粮</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>cao_cao</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>ruler</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>logistics</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>logistics</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>核对军粮簿册、巡查仓储并补正调拨缺漏，确保下月军需可按时发出。</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>以巡察为主推进仓储清点，本月达成军粮账目闭合。</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>1</v>
+      </c>
+      <c r="L3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>logistics_balanced</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>current_value:8</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>current_value:11</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>merit:7|fame:0|trust:0|success_note:军粮条目核实清楚，幕府记你一功。</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>merit:3|fame:1|trust:0|success_note:仓储漏洞一并补齐，本月后勤事务完成得尤为稳妥。</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>merit_delta:0|fame_delta:0|trust_delta:0|failure_note:账簿仍有漏项，军粮事务虽未酿祸，但未能立功。</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="T3" t="n">
+        <v>20</v>
+      </c>
+      <c r="U3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>task_clan_pacify</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>安抚宗族</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>cao_cao</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>ruler</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>politics</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>politics_basic</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>走访城中有势力的宗族与里正，厘清近期征调与治安摩擦，稳住地方人心。</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>以拜访为主缓和地方张力，兼顾基础政务沟通。</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>clan_pacify_social</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>current_value:8</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>current_value:11</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>merit:5|fame:1|trust:1|success_note:地方宗族情绪稍稳，主君记你善于斡旋。</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>merit:2|fame:1|trust:1|success_note:城中宗族争执一并压住，你在地方层面的可信度明显提升。</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>merit_delta:0|fame_delta:0|trust_delta:-1|failure_note:安抚效果有限，地方仍有不满之声。</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>politics_mid</t>
+        </is>
+      </c>
+      <c r="T4" t="n">
+        <v>40</v>
+      </c>
+      <c r="U4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>task_recommend_talent</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>举荐人才</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>cao_cao</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>ruler</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>personnel</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>personnel</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H5" t="n">
+        <v>3</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>接触可用士人，汇总才干与来历，为幕府下一轮用人提供名单。</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>以拜访与读书配合，整理可供举荐的人才脉络。</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>1</v>
+      </c>
+      <c r="L5" t="n">
+        <v>2</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>recommend_talent_network</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>current_value:7</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>current_value:10</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>merit:6|fame:1|trust:1|success_note:举荐脉络清楚，主君认可你在识人上的用心。</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>merit:3|fame:2|trust:1|success_note:所荐之才颇有条理，幕府对你的人脉判断更为看重。</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>merit_delta:0|fame_delta:0|trust_delta:0|failure_note:候选名单零散，本月未形成可用的人事建议。</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>politics_mid|dispatch</t>
+        </is>
+      </c>
+      <c r="T5" t="n">
+        <v>60</v>
+      </c>
+      <c r="U5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>tier</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>unlock_task_tags</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>blocked_task_tags</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>merit_threshold</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>next_office_id</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>prev_office_id</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>address_title</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>stipend_text</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>is_phase2_1_available</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>sort_order</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>office_commoner</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>白身</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>尚未正式入仕，只能通过零散事务证明自己可被纳入幕府秩序。</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>logistics</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>admin|politics_basic|politics_mid|dispatch</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>office_congshi</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>布衣</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>暂无正式俸给，以临时差事建立功绩。</t>
+        </is>
+      </c>
+      <c r="L2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>office_congshi</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>从事</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>正式进入势力政务链条的基础幕僚官，开始接受月度考评与正式事务指派。</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>logistics|admin|politics_basic</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>central_affairs</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>10</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>office_zhubu</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>office_commoner</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>从事君</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>列属幕府，食禄有定，须以月度公事自证才干。</t>
+        </is>
+      </c>
+      <c r="L3" t="b">
+        <v>1</v>
+      </c>
+      <c r="M3" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>office_zhubu</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>主簿级辅官</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>可直接接触更稳定的内政与人事事务，开始拥有更明确的政治可见度。</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>logistics|admin|politics_basic|personnel|politics_mid|dispatch</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="n">
+        <v>25</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>office_central_aide</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>office_congshi</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>主簿</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>秉掌案牍与调度，已入可被主君直接考察的辅官序列。</t>
+        </is>
+      </c>
+      <c r="L4" t="b">
+        <v>1</v>
+      </c>
+      <c r="M4" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>office_central_aide</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>中枢佐官</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>开始接触势力中枢决策与高级人事安排，成为政治运转中的稳定节点。</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>admin|personnel|politics_mid|dispatch|central_affairs</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="n">
+        <v>40</v>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>office_zhubu</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>中枢佐官</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>参与更高层的幕府事务，已被视作可长期培养的核心幕僚。</t>
+        </is>
+      </c>
+      <c r="L5" t="b">
+        <v>1</v>
+      </c>
+      <c r="M5" t="n">
+        <v>30</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>